<commit_message>
Make portfolio fully reproducible with public data
</commit_message>
<xml_diff>
--- a/deliverables/Distributor_Case_Study_Analysis.xlsx
+++ b/deliverables/Distributor_Case_Study_Analysis.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual Trend" sheetId="1" r:id="R897d596f69324036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Profitability" sheetId="2" r:id="Ra9dd77eb94fb4e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concentration" sheetId="3" r:id="Rba99e5ff1378426e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retention Summary" sheetId="4" r:id="R74cd5a7d677646dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="5" r:id="R27eca8ec218448b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Growth" sheetId="6" r:id="R08d49ee0e7ad44e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Concentration" sheetId="7" r:id="R90d97107baa04421"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retention by Segment" sheetId="8" r:id="R108d87cf0d314195"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach Priorities" sheetId="9" r:id="Raeeae03ff0f54934"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="10" r:id="R4239222555064c97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual Trend" sheetId="1" r:id="R7bd47d05818b4891"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Profitability" sheetId="2" r:id="Rf75438bc8fe94fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concentration" sheetId="3" r:id="Rb8d85b9ad7a646cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retention Summary" sheetId="4" r:id="R735dcf526526478c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="5" r:id="R32af9654d69c4455"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Growth" sheetId="6" r:id="R5bf8447856974af0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Concentration" sheetId="7" r:id="R421d4145eff84158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retention by Segment" sheetId="8" r:id="R1d62f2ec6b7d4fde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach Priorities" sheetId="9" r:id="Rfd5fa5eb1d6e48c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="10" r:id="Rd317184595514f47"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -400,7 +400,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3ac7a94d7b8a4450"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7fc75f3e77a44247"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1122,9 +1122,9 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R658c2c9457b54ae2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11ee65490b4241f2"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d7f6187c185488f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2567eacb13324040"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1770,7 +1770,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6733247f55b54c74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0670476e14044a76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4476,7 +4476,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c13abd3447d43a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R635cbaea59fc46b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7504,7 +7504,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d73844fc6ec4ca9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dd6bb881abf483a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7711,7 +7711,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4b836cb36fe46a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43626205f5944b10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10841,7 +10841,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5f81c1b4f1c4c3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc07ff804437344b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12371,7 +12371,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01a1898282c14603"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd9087b3f6434973"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14881,7 +14881,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb0e4e6b37c84cc0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R859d9307ece14446"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17239,7 +17239,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06911b8818ee46ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ce8fb4098d542b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>